<commit_message>
Troca do Modelo_Açoes e Adicição de requirements
</commit_message>
<xml_diff>
--- a/assets/Modelo_Acoes.xlsx
+++ b/assets/Modelo_Acoes.xlsx
@@ -139,15 +139,21 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -155,19 +161,37 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -496,37 +520,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29">
-      <c r="A1" s="2"/>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-      <c r="I1" s="2"/>
-      <c r="J1" s="2"/>
-      <c r="K1" s="2"/>
-      <c r="L1" s="2"/>
-      <c r="M1" s="2"/>
-      <c r="N1" s="2"/>
-      <c r="O1" s="2"/>
-      <c r="P1" s="2"/>
-      <c r="Q1" s="2"/>
-      <c r="R1" s="2"/>
-      <c r="S1" s="2"/>
-      <c r="T1" s="2"/>
-      <c r="U1" s="2"/>
-      <c r="V1" s="2"/>
-      <c r="W1" s="2"/>
-      <c r="X1" s="1" t="s">
+      <c r="A1" s="1"/>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
+      <c r="O1" s="1"/>
+      <c r="P1" s="1"/>
+      <c r="Q1" s="1"/>
+      <c r="R1" s="1"/>
+      <c r="S1" s="1"/>
+      <c r="T1" s="1"/>
+      <c r="U1" s="1"/>
+      <c r="V1" s="1"/>
+      <c r="W1" s="1"/>
+      <c r="X1" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="Y1" s="1"/>
-      <c r="Z1" s="2"/>
-      <c r="AA1" s="2"/>
-      <c r="AB1" s="2"/>
-      <c r="AC1" s="2"/>
+      <c r="Y1" s="4"/>
+      <c r="Z1" s="1"/>
+      <c r="AA1" s="1"/>
+      <c r="AB1" s="1"/>
+      <c r="AC1" s="1"/>
     </row>
     <row r="2" spans="1:29">
       <c r="A2" s="2" t="s">

</xml_diff>